<commit_message>
added api checking, made changes to mroe stuff like the alias
</commit_message>
<xml_diff>
--- a/output/pdf_financials_xlsx/AAAJ.P.xlsx
+++ b/output/pdf_financials_xlsx/AAAJ.P.xlsx
@@ -6469,7 +6469,11 @@
           <t>Proceeds from share issuances</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>CommonStockIssuance</t>
+        </is>
+      </c>
       <c r="E74" s="5" t="n">
         <v>0.235</v>
       </c>

</xml_diff>